<commit_message>
Add initial implementation of xcorr assessment, fix issues with calcing pred_adj
</commit_message>
<xml_diff>
--- a/data/HighTideOutlookStationList_05_17_23_PAC_SLT.xlsx
+++ b/data/HighTideOutlookStationList_05_17_23_PAC_SLT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\high_tide_flooding\Seasonal_High_Tide_Flooding_Prediction\station list\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matthew.conlin\Documents\Projects\CORA-HTF\HTF\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EADD35-82C6-4C87-8C87-E1128E159D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A0B3A7-2774-4BCE-8050-4A951BAC33A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -424,6 +424,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -484,7 +487,7 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -508,19 +511,10 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -557,7 +551,23 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -844,19 +854,19 @@
   <dimension ref="A1:J113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="21" customWidth="1"/>
-    <col min="2" max="2" width="33.85546875" style="23" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="21.7109375" style="10" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" style="10" customWidth="1"/>
-    <col min="9" max="10" width="9.140625" style="10"/>
+    <col min="1" max="1" width="13.5703125" style="18" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" style="20" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="21.7109375" style="9" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" style="9" customWidth="1"/>
+    <col min="9" max="10" width="9.140625" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -891,3580 +901,3580 @@
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="26">
         <v>21.954444444444398</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="26">
         <v>-159.35611111111101</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F2" s="8">
+      <c r="E2" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="23">
         <v>1.9596</v>
       </c>
       <c r="H2" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J2" s="10">
+      <c r="J2" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
+      <c r="A3" s="10">
         <v>1612340</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="27">
         <v>21.306699999999999</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="27">
         <v>-157.86699999999999</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="8">
+      <c r="E3" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F3" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="23">
         <v>1.7514000000000001</v>
       </c>
       <c r="H3" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J3" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="11">
+      <c r="A4" s="10">
         <v>1612480</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="27">
         <v>21.433055555555502</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="27">
         <v>-157.79</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F4" s="8">
+      <c r="E4" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="23">
         <v>2.2496999999999998</v>
       </c>
       <c r="H4" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="11">
+      <c r="A5" s="10">
         <v>1615680</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="27">
         <v>20.895</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="27">
         <v>-156.47666666666601</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F5" s="8">
+      <c r="E5" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="23">
         <v>2.1741000000000001</v>
       </c>
       <c r="H5" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+      <c r="A6" s="10">
         <v>1617433</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="27">
         <v>20.036583333280301</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="27">
         <v>-155.82936111132301</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F6" s="8">
+      <c r="E6" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="23">
         <v>3.5097</v>
       </c>
       <c r="H6" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>1617760</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="27">
         <v>19.730277777777701</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="27">
         <v>-155.055833333333</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F7" s="8">
+      <c r="E7" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="23">
         <v>2.5768</v>
       </c>
       <c r="H7" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
+      <c r="A8" s="10">
         <v>1619910</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="27">
         <v>28.2117</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="27">
         <v>-177.36</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F8" s="8">
+      <c r="E8" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F8" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="23">
         <v>3.5556000000000001</v>
       </c>
       <c r="H8" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J8" s="9">
         <v>-11</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="11">
+      <c r="A9" s="10">
         <v>1630000</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="27">
         <v>13.43872</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="27">
         <v>144.65394444439099</v>
       </c>
-      <c r="E9" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F9" s="8">
+      <c r="E9" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F9" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="24">
         <v>5.0106000000000002</v>
       </c>
       <c r="H9" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="9">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
+      <c r="A10" s="10">
         <v>1770000</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="27">
         <v>-14.28</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="27">
         <v>-170.69</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="F10" s="8">
+      <c r="E10" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="F10" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="23">
         <v>20.1035</v>
       </c>
       <c r="H10" s="7">
         <v>2015.5</v>
       </c>
-      <c r="I10" s="14" t="s">
+      <c r="I10" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="9">
         <v>-11</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="11">
+      <c r="A11" s="10">
         <v>1820000</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="27">
         <v>8.7316099999999999</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="27">
         <v>167.736222222116</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F11" s="8">
+      <c r="E11" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="23">
         <v>3.2799</v>
       </c>
       <c r="H11" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="9">
         <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
+      <c r="A12" s="10">
         <v>1890000</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="27">
         <v>19.29</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="27">
         <v>166.61799999999999</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F12" s="8">
+      <c r="E12" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" s="22">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="23">
         <v>2.4735999999999998</v>
       </c>
       <c r="H12" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J12" s="10">
+      <c r="J12" s="9">
         <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="11">
+      <c r="A13" s="10">
         <v>8413320</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="27">
         <v>44.3917</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="27">
         <v>-68.204999999999998</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F13" s="8">
+      <c r="E13" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" s="22">
         <v>0.63863999999999965</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="23">
         <v>2.4163000000000001</v>
       </c>
       <c r="H13" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J13" s="10">
+      <c r="J13" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="11">
+      <c r="A14" s="10">
         <v>8418150</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="27">
         <v>43.656700000000001</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="27">
         <v>-70.246700000000004</v>
       </c>
-      <c r="E14" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F14" s="8">
+      <c r="E14" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F14" s="22">
         <v>0.62076204000000024</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="23">
         <v>1.7519</v>
       </c>
       <c r="H14" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J14" s="10">
+      <c r="J14" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="12">
         <v>8443970</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="27">
         <v>42.354799999999997</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="27">
         <v>-71.053399999999996</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="22">
         <v>0.6803866097560971</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="22">
         <v>0.62522356000000001</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="23">
         <v>3.4363999999999999</v>
       </c>
       <c r="H15" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J15" s="10">
+      <c r="J15" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="12">
         <v>8447930</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="27">
         <v>41.523299999999999</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="27">
         <v>-70.671700000000001</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="22">
         <v>1.0044872682926833</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="22">
         <v>0.52689368000000003</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="23">
         <v>3.9066000000000001</v>
       </c>
       <c r="H16" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I16" s="10" t="s">
+      <c r="I16" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J16" s="10">
+      <c r="J16" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="12">
         <v>8449130</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="27">
         <v>41.284999999999997</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="27">
         <v>-70.096699999999998</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="22">
         <v>0.74018029268292684</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="22">
         <v>0.54356351999999997</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="23">
         <v>4.5705</v>
       </c>
       <c r="H17" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="I17" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J17" s="10">
+      <c r="J17" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="12">
         <v>8452660</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="27">
         <v>41.505000000000003</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="27">
         <v>-71.326700000000002</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="22">
         <v>0.80781731707317106</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="22">
         <v>0.54695559999999999</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="23">
         <v>3.58</v>
       </c>
       <c r="H18" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J18" s="10">
+      <c r="J18" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="11">
+      <c r="A19" s="10">
         <v>8454000</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="27">
         <v>41.807099999999998</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="27">
         <v>-71.401200000000003</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="22">
         <v>0.65827834146341457</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="22">
         <v>0.5590347200000001</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="23">
         <v>3.5874000000000001</v>
       </c>
       <c r="H19" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J19" s="10">
+      <c r="J19" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="16">
+      <c r="A20" s="13">
         <v>8461490</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="27">
         <v>41.361388888888797</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="27">
         <v>-72.089972222222201</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="22">
         <v>0.59448724390243912</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="22">
         <v>0.53719611999999994</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="23">
         <v>4.1554000000000002</v>
       </c>
       <c r="H20" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I20" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J20" s="10">
+      <c r="J20" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="12">
         <v>8467150</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="27">
         <v>41.173299999999998</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="27">
         <v>-73.181700000000006</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="22">
         <v>0.482414634146342</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="22">
         <v>0.58924000000000021</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="23">
         <v>3.8102</v>
       </c>
       <c r="H21" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="I21" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J21" s="10">
+      <c r="J21" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="16">
+      <c r="A22" s="13">
         <v>8510560</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="27">
         <v>41.048299999999998</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="27">
         <v>-71.959999999999994</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="22">
         <v>0.60195121951219521</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="22">
         <v>0.53080000000000016</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="23">
         <v>4.8769</v>
       </c>
       <c r="H22" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="I22" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J22" s="10">
+      <c r="J22" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="23" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
+      <c r="A23" s="14">
         <v>8516945</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="23">
         <v>40.810299999999998</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="23">
         <v>-73.764899999999997</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="23">
         <v>0.51634146341463438</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="23">
         <v>0.59512000000000009</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="23">
         <v>3.1484999999999999</v>
       </c>
       <c r="H23" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I23" s="10" t="s">
+      <c r="I23" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J23" s="14">
+      <c r="J23" s="11">
         <v>-5</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="12">
         <v>8518750</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="27">
         <v>40.700600000000001</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="27">
         <v>-74.014200000000002</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="22">
         <v>0.65399999999999969</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="22">
         <v>0.56163999999999992</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="23">
         <v>4.0518999999999998</v>
       </c>
       <c r="H24" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="I24" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J24" s="10">
+      <c r="J24" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="16">
+      <c r="A25" s="13">
         <v>8519483</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="12">
+      <c r="C25" s="27">
         <v>40.636699999999998</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="27">
         <v>-74.1417</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="22">
         <v>0.51512195121951221</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="22">
         <v>0.56720000000000015</v>
       </c>
-      <c r="G25" s="14">
+      <c r="G25" s="23">
         <v>4.2508999999999997</v>
       </c>
       <c r="H25" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J25" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="11">
+      <c r="A26" s="10">
         <v>8531680</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="12">
+      <c r="C26" s="27">
         <v>40.466900000000003</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="27">
         <v>-74.009399999999999</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="22">
         <v>0.45022492682926862</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="22">
         <v>0.56369832000000009</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="23">
         <v>4.7683</v>
       </c>
       <c r="H26" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J26" s="10">
+      <c r="J26" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="11">
+      <c r="A27" s="10">
         <v>8534720</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="27">
         <v>39.354999999999997</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="27">
         <v>-74.418300000000002</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="22">
         <v>0.42625129268292716</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="22">
         <v>0.55612068000000003</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="23">
         <v>5.0511999999999997</v>
       </c>
       <c r="H27" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I27" s="10" t="s">
+      <c r="I27" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J27" s="10">
+      <c r="J27" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="16">
+      <c r="A28" s="13">
         <v>8536110</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C28" s="12">
+      <c r="C28" s="27">
         <v>38.968333333333298</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="27">
         <v>-74.959999999999994</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="22">
         <v>0.38268292682926841</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="22">
         <v>0.56639999999999979</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28" s="23">
         <v>5.7545999999999999</v>
       </c>
       <c r="H28" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I28" s="10" t="s">
+      <c r="I28" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J28" s="10">
+      <c r="J28" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="29" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11">
+      <c r="A29" s="10">
         <v>8545240</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="27">
         <v>39.933333333333302</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="27">
         <v>-75.141666666666595</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="23">
         <v>0.46099999999999985</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="23">
         <v>0.58156000000000008</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="23">
         <v>4.6144999999999996</v>
       </c>
       <c r="H29" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I29" s="10" t="s">
+      <c r="I29" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J29" s="14">
+      <c r="J29" s="11">
         <v>-5</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="11">
+      <c r="A30" s="10">
         <v>8551910</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="27">
         <v>39.558305555555499</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="27">
         <v>-75.573305555555507</v>
       </c>
-      <c r="E30" s="8">
+      <c r="E30" s="22">
         <v>0.41512195121951256</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="22">
         <v>0.57120000000000015</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="23">
         <v>4.3619000000000003</v>
       </c>
       <c r="H30" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I30" s="10" t="s">
+      <c r="I30" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J30" s="10">
+      <c r="J30" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="11">
+      <c r="A31" s="10">
         <v>8557380</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="27">
         <v>38.781694444444398</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="27">
         <v>-75.12</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31" s="22">
         <v>0.41101229268292694</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F31" s="22">
         <v>0.55673024000000004</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="23">
         <v>4.7496999999999998</v>
       </c>
       <c r="H31" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I31" s="10" t="s">
+      <c r="I31" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J31" s="10">
+      <c r="J31" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="16">
+      <c r="A32" s="13">
         <v>8571892</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="27">
         <v>38.573300000000003</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="27">
         <v>-76.068299999999994</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32" s="22">
         <v>0.44518417073170746</v>
       </c>
-      <c r="F32" s="8">
+      <c r="F32" s="22">
         <v>0.52487555999999991</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32" s="23">
         <v>4.6577000000000002</v>
       </c>
       <c r="H32" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I32" s="10" t="s">
+      <c r="I32" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J32" s="10">
+      <c r="J32" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="11">
+      <c r="A33" s="10">
         <v>8573364</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="27">
         <v>39.213329999999999</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="27">
         <v>-76.245000000000005</v>
       </c>
-      <c r="E33" s="8">
+      <c r="E33" s="22">
         <v>0.54007317073170746</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="22">
         <v>0.52107999999999999</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33" s="23">
         <v>4.8030999999999997</v>
       </c>
       <c r="H33" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I33" s="10" t="s">
+      <c r="I33" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J33" s="10">
+      <c r="J33" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="12">
         <v>8574680</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="27">
         <v>39.266669999999998</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="27">
         <v>-76.578333333333305</v>
       </c>
-      <c r="E34" s="8">
+      <c r="E34" s="22">
         <v>0.40854614634146336</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="22">
         <v>0.52024352000000018</v>
       </c>
-      <c r="G34" s="9">
+      <c r="G34" s="23">
         <v>3.9359000000000002</v>
       </c>
       <c r="H34" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I34" s="10" t="s">
+      <c r="I34" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J34" s="10">
+      <c r="J34" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
+      <c r="A35" s="12">
         <v>8575512</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="27">
         <v>38.983280000000001</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="27">
         <v>-76.481555555131706</v>
       </c>
-      <c r="E35" s="8">
+      <c r="E35" s="22">
         <v>0.29370731707317077</v>
       </c>
-      <c r="F35" s="8">
+      <c r="F35" s="22">
         <v>0.51751999999999998</v>
       </c>
-      <c r="G35" s="9">
+      <c r="G35" s="23">
         <v>4.4093</v>
       </c>
       <c r="H35" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I35" s="10" t="s">
+      <c r="I35" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J35" s="10">
+      <c r="J35" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="11">
+      <c r="A36" s="10">
         <v>8577330</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="27">
         <v>38.316670000000002</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="27">
         <v>-76.451666666666597</v>
       </c>
-      <c r="E36" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F36" s="8">
+      <c r="E36" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F36" s="22">
         <v>0.51797355999999994</v>
       </c>
-      <c r="G36" s="9">
+      <c r="G36" s="23">
         <v>5.5438000000000001</v>
       </c>
       <c r="H36" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I36" s="10" t="s">
+      <c r="I36" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J36" s="10">
+      <c r="J36" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="11">
+      <c r="A37" s="10">
         <v>8594900</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="27">
         <v>38.873330000000003</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="27">
         <v>-77.021666666666604</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E37" s="22">
         <v>0.31538280487804893</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="22">
         <v>0.53860419999999998</v>
       </c>
-      <c r="G37" s="9">
+      <c r="G37" s="23">
         <v>4.2537000000000003</v>
       </c>
       <c r="H37" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I37" s="10" t="s">
+      <c r="I37" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J37" s="10">
+      <c r="J37" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="11">
+      <c r="A38" s="10">
         <v>8631044</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="27">
         <v>37.607777777777699</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="27">
         <v>-75.685833333333306</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E38" s="22">
         <v>0.60670731707317094</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="22">
         <v>0.55500000000000016</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="23">
         <v>5.2598000000000003</v>
       </c>
       <c r="H38" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I38" s="10" t="s">
+      <c r="I38" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J38" s="10">
+      <c r="J38" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="16">
+      <c r="A39" s="13">
         <v>8632200</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="27">
         <v>37.165190000000003</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="27">
         <v>-75.988444444338398</v>
       </c>
-      <c r="E39" s="8">
+      <c r="E39" s="22">
         <v>0.47642121951219529</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="22">
         <v>0.5358212</v>
       </c>
-      <c r="G39" s="9">
+      <c r="G39" s="23">
         <v>4.5861999999999998</v>
       </c>
       <c r="H39" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I39" s="10" t="s">
+      <c r="I39" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J39" s="10">
+      <c r="J39" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="11">
+      <c r="A40" s="10">
         <v>8635750</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="27">
         <v>37.996111111111098</v>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="27">
         <v>-76.464444444444396</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E40" s="22">
         <v>0.45623614634146337</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F40" s="22">
         <v>0.51833591999999995</v>
       </c>
-      <c r="G40" s="9">
+      <c r="G40" s="23">
         <v>6.6184000000000003</v>
       </c>
       <c r="H40" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I40" s="10" t="s">
+      <c r="I40" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J40" s="10">
+      <c r="J40" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="11">
+      <c r="A41" s="10">
         <v>8636580</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="27">
         <v>37.616199999999999</v>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="27">
         <v>-76.290000000000006</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E41" s="22">
         <v>0.49</v>
       </c>
-      <c r="F41" s="8">
+      <c r="F41" s="22">
         <v>0.52</v>
       </c>
-      <c r="G41" s="9">
+      <c r="G41" s="23">
         <v>7.3681000000000001</v>
       </c>
       <c r="H41" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I41" s="10" t="s">
+      <c r="I41" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J41" s="10">
+      <c r="J41" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="11">
+      <c r="A42" s="10">
         <v>8638610</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="12">
+      <c r="C42" s="27">
         <v>36.946666666666601</v>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="27">
         <v>-76.33</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E42" s="22">
         <v>0.53195121951219515</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F42" s="22">
         <v>0.53360000000000007</v>
       </c>
-      <c r="G42" s="9">
+      <c r="G42" s="23">
         <v>5.7567000000000004</v>
       </c>
       <c r="H42" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I42" s="10" t="s">
+      <c r="I42" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="J42" s="10">
+      <c r="J42" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="11">
+      <c r="A43" s="10">
         <v>8651370</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="12">
+      <c r="C43" s="27">
         <v>36.183305555555499</v>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="27">
         <v>-75.746694444444401</v>
       </c>
-      <c r="E43" s="8">
+      <c r="E43" s="22">
         <v>0.5530472682926828</v>
       </c>
-      <c r="F43" s="8">
+      <c r="F43" s="22">
         <v>0.54495128000000004</v>
       </c>
-      <c r="G43" s="9">
+      <c r="G43" s="23">
         <v>4.5171999999999999</v>
       </c>
       <c r="H43" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I43" s="10" t="s">
+      <c r="I43" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J43" s="10">
+      <c r="J43" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="18">
+      <c r="A44" s="15">
         <v>8652587</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C44" s="14">
+      <c r="C44" s="23">
         <v>35.795000000000002</v>
       </c>
-      <c r="D44" s="14">
+      <c r="D44" s="23">
         <v>-75.548299999999998</v>
       </c>
-      <c r="E44" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="F44" s="9">
+      <c r="E44" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="F44" s="23">
         <v>0.51440000000000008</v>
       </c>
-      <c r="G44" s="9">
+      <c r="G44" s="23">
         <v>6.4757999999999996</v>
       </c>
       <c r="H44" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I44" s="14" t="s">
+      <c r="I44" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="J44" s="10">
+      <c r="J44" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="11">
+      <c r="A45" s="10">
         <v>8656483</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="12">
+      <c r="C45" s="27">
         <v>34.72</v>
       </c>
-      <c r="D45" s="12">
+      <c r="D45" s="27">
         <v>-76.67</v>
       </c>
-      <c r="E45" s="8">
+      <c r="E45" s="22">
         <v>0.29324421951219515</v>
       </c>
-      <c r="F45" s="8">
+      <c r="F45" s="22">
         <v>0.54314828000000004</v>
       </c>
-      <c r="G45" s="9">
+      <c r="G45" s="23">
         <v>4.6853999999999996</v>
       </c>
       <c r="H45" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I45" s="10" t="s">
+      <c r="I45" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J45" s="10">
+      <c r="J45" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="15">
+      <c r="A46" s="12">
         <v>8658120</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C46" s="12">
+      <c r="C46" s="27">
         <v>34.226700000000001</v>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="27">
         <v>-77.953299999999999</v>
       </c>
-      <c r="E46" s="8">
+      <c r="E46" s="22">
         <v>0.24982926829268304</v>
       </c>
-      <c r="F46" s="8">
+      <c r="F46" s="22">
         <v>0.55708000000000002</v>
       </c>
-      <c r="G46" s="9">
+      <c r="G46" s="23">
         <v>4.0648999999999997</v>
       </c>
       <c r="H46" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I46" s="10" t="s">
+      <c r="I46" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J46" s="10">
+      <c r="J46" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="11">
+      <c r="A47" s="10">
         <v>8661070</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C47" s="12">
+      <c r="C47" s="27">
         <v>33.655000000000001</v>
       </c>
-      <c r="D47" s="12">
+      <c r="D47" s="27">
         <v>-78.918300000000002</v>
       </c>
-      <c r="E47" s="8">
+      <c r="E47" s="22">
         <v>0.57958536585365961</v>
       </c>
-      <c r="F47" s="8">
+      <c r="F47" s="22">
         <v>0.56828000000000012</v>
       </c>
-      <c r="G47" s="9">
+      <c r="G47" s="23">
         <v>3.2917999999999998</v>
       </c>
       <c r="H47" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I47" s="10" t="s">
+      <c r="I47" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J47" s="10">
+      <c r="J47" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="15">
+      <c r="A48" s="12">
         <v>8665530</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="12">
+      <c r="C48" s="27">
         <v>32.781700000000001</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="27">
         <v>-79.924999999999997</v>
       </c>
-      <c r="E48" s="8">
+      <c r="E48" s="22">
         <v>0.37679034146341461</v>
       </c>
-      <c r="F48" s="8">
+      <c r="F48" s="22">
         <v>0.5702942400000004</v>
       </c>
-      <c r="G48" s="9">
+      <c r="G48" s="23">
         <v>4.2732000000000001</v>
       </c>
       <c r="H48" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I48" s="10" t="s">
+      <c r="I48" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J48" s="10">
+      <c r="J48" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="15">
+      <c r="A49" s="12">
         <v>8670870</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C49" s="12">
+      <c r="C49" s="27">
         <v>32.033299999999997</v>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="27">
         <v>-80.901700000000005</v>
       </c>
-      <c r="E49" s="8">
+      <c r="E49" s="22">
         <v>0.45658643902439033</v>
       </c>
-      <c r="F49" s="8">
+      <c r="F49" s="22">
         <v>0.59149264000000024</v>
       </c>
-      <c r="G49" s="9">
+      <c r="G49" s="23">
         <v>4.7576000000000001</v>
       </c>
       <c r="H49" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I49" s="10" t="s">
+      <c r="I49" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J49" s="10">
+      <c r="J49" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="19">
+      <c r="A50" s="16">
         <v>8720030</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C50" s="12">
+      <c r="C50" s="27">
         <v>30.671700000000001</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="27">
         <v>-81.465000000000003</v>
       </c>
-      <c r="E50" s="8">
+      <c r="E50" s="22">
         <v>0.59246341463414676</v>
       </c>
-      <c r="F50" s="8">
+      <c r="F50" s="22">
         <v>0.57996000000000003</v>
       </c>
-      <c r="G50" s="9">
+      <c r="G50" s="23">
         <v>3.464</v>
       </c>
       <c r="H50" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I50" s="10" t="s">
+      <c r="I50" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J50" s="10">
+      <c r="J50" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="51" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="19">
+      <c r="A51" s="16">
         <v>8720218</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="23">
         <v>30.396699999999999</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="23">
         <v>-81.430000000000007</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="23">
         <v>0.443</v>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="23">
         <v>0.56031999999999993</v>
       </c>
-      <c r="G51" s="9">
+      <c r="G51" s="23">
         <v>4.1310000000000002</v>
       </c>
       <c r="H51" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I51" s="10" t="s">
+      <c r="I51" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J51" s="14">
+      <c r="J51" s="11">
         <v>-5</v>
       </c>
     </row>
     <row r="52" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="19">
+      <c r="A52" s="16">
         <v>8721604</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52" s="23">
         <v>28.415800000000001</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="23">
         <v>-80.593100000000007</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="23">
         <v>0.63626829268292728</v>
       </c>
-      <c r="F52" s="9">
+      <c r="F52" s="23">
         <v>0.54771999999999998</v>
       </c>
-      <c r="G52" s="9">
+      <c r="G52" s="23">
         <v>6.2511999999999999</v>
       </c>
       <c r="H52" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I52" s="10" t="s">
+      <c r="I52" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J52" s="14">
+      <c r="J52" s="11">
         <v>-5</v>
       </c>
     </row>
     <row r="53" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="19">
+      <c r="A53" s="16">
         <v>8723214</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C53" s="9">
+      <c r="C53" s="23">
         <v>25.731400000000001</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D53" s="23">
         <v>-80.161799999999999</v>
       </c>
-      <c r="E53" s="9">
+      <c r="E53" s="23">
         <v>0.40007317073170756</v>
       </c>
-      <c r="F53" s="9">
+      <c r="F53" s="23">
         <v>0.52668000000000004</v>
       </c>
-      <c r="G53" s="9">
+      <c r="G53" s="23">
         <v>4.1174999999999997</v>
       </c>
       <c r="H53" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I53" s="10" t="s">
+      <c r="I53" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J53" s="14">
+      <c r="J53" s="11">
         <v>-5</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" s="19">
+      <c r="A54" s="16">
         <v>8723970</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C54" s="12">
+      <c r="C54" s="27">
         <v>24.7117</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="27">
         <v>-81.105000000000004</v>
       </c>
-      <c r="E54" s="8">
+      <c r="E54" s="22">
         <v>0.5871463414634146</v>
       </c>
-      <c r="F54" s="8">
+      <c r="F54" s="22">
         <v>0.51188</v>
       </c>
-      <c r="G54" s="9">
+      <c r="G54" s="23">
         <v>4.7962999999999996</v>
       </c>
       <c r="H54" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I54" s="10" t="s">
+      <c r="I54" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J54" s="10">
+      <c r="J54" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="19">
+      <c r="A55" s="16">
         <v>8724580</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C55" s="12">
+      <c r="C55" s="27">
         <v>24.555700000000002</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="27">
         <v>-81.807900000000004</v>
       </c>
-      <c r="E55" s="8">
+      <c r="E55" s="22">
         <v>0.33283234146341478</v>
       </c>
-      <c r="F55" s="8">
+      <c r="F55" s="22">
         <v>0.52205255999999989</v>
       </c>
-      <c r="G55" s="9">
+      <c r="G55" s="23">
         <v>3.7170000000000001</v>
       </c>
       <c r="H55" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I55" s="10" t="s">
+      <c r="I55" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J55" s="10">
+      <c r="J55" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="19">
+      <c r="A56" s="16">
         <v>8725110</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C56" s="12">
+      <c r="C56" s="27">
         <v>26.131699999999999</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="27">
         <v>-81.807500000000005</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56" s="22">
         <v>0.3455121951219513</v>
       </c>
-      <c r="F56" s="8">
+      <c r="F56" s="22">
         <v>0.5349600000000001</v>
       </c>
-      <c r="G56" s="9">
+      <c r="G56" s="23">
         <v>4.2851999999999997</v>
       </c>
       <c r="H56" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I56" s="10" t="s">
+      <c r="I56" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J56" s="10">
+      <c r="J56" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="18">
+      <c r="A57" s="15">
         <v>8725520</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C57" s="14">
+      <c r="C57" s="23">
         <v>26.6477</v>
       </c>
-      <c r="D57" s="14">
+      <c r="D57" s="23">
         <v>-81.871200000000002</v>
       </c>
-      <c r="E57" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="F57" s="9">
+      <c r="E57" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="F57" s="23">
         <v>0.51604000000000005</v>
       </c>
-      <c r="G57" s="9">
+      <c r="G57" s="23">
         <v>4.1752000000000002</v>
       </c>
       <c r="H57" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I57" s="14" t="s">
+      <c r="I57" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="J57" s="10">
+      <c r="J57" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" s="19">
+      <c r="A58" s="16">
         <v>8726520</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C58" s="12">
+      <c r="C58" s="27">
         <v>27.7606</v>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="27">
         <v>-82.626900000000006</v>
       </c>
-      <c r="E58" s="8">
+      <c r="E58" s="22">
         <v>0.83596024390243906</v>
       </c>
-      <c r="F58" s="8">
+      <c r="F58" s="22">
         <v>0.52753720000000015</v>
       </c>
-      <c r="G58" s="9">
+      <c r="G58" s="23">
         <v>4.1295999999999999</v>
       </c>
       <c r="H58" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I58" s="10" t="s">
+      <c r="I58" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J58" s="10">
+      <c r="J58" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="19">
+      <c r="A59" s="16">
         <v>8726724</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C59" s="12">
+      <c r="C59" s="27">
         <v>27.978000000000002</v>
       </c>
-      <c r="D59" s="12">
+      <c r="D59" s="27">
         <v>-82.831999999999994</v>
       </c>
-      <c r="E59" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F59" s="8">
+      <c r="E59" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F59" s="22">
         <v>0.53363999999999989</v>
       </c>
-      <c r="G59" s="9">
+      <c r="G59" s="23">
         <v>4.8956</v>
       </c>
       <c r="H59" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I59" s="10" t="s">
+      <c r="I59" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J59" s="10">
+      <c r="J59" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="18">
+      <c r="A60" s="15">
         <v>8727520</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C60" s="14">
+      <c r="C60" s="23">
         <v>29.135000000000002</v>
       </c>
-      <c r="D60" s="14">
+      <c r="D60" s="23">
         <v>-83.031700000000001</v>
       </c>
-      <c r="E60" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="F60" s="9">
+      <c r="E60" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="F60" s="23">
         <v>0.54632000000000014</v>
       </c>
-      <c r="G60" s="9">
+      <c r="G60" s="23">
         <v>3.7528000000000001</v>
       </c>
       <c r="H60" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I60" s="14" t="s">
+      <c r="I60" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="J60" s="10">
+      <c r="J60" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="19">
+      <c r="A61" s="16">
         <v>8728690</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C61" s="12">
+      <c r="C61" s="27">
         <v>29.726700000000001</v>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="27">
         <v>-84.981700000000004</v>
       </c>
-      <c r="E61" s="8">
+      <c r="E61" s="22">
         <v>0.42259914634146345</v>
       </c>
-      <c r="F61" s="8">
+      <c r="F61" s="22">
         <v>0.51968140000000007</v>
       </c>
-      <c r="G61" s="9">
+      <c r="G61" s="23">
         <v>3.7118000000000002</v>
       </c>
       <c r="H61" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I61" s="10" t="s">
+      <c r="I61" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J61" s="10">
+      <c r="J61" s="9">
         <v>-5</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="19">
+      <c r="A62" s="16">
         <v>8729108</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C62" s="12">
+      <c r="C62" s="27">
         <v>30.152277777777702</v>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="27">
         <v>-85.666944444444397</v>
       </c>
-      <c r="E62" s="8">
+      <c r="E62" s="22">
         <v>0.35319512195121949</v>
       </c>
-      <c r="F62" s="8">
+      <c r="F62" s="22">
         <v>0.51636000000000004</v>
       </c>
-      <c r="G62" s="9">
+      <c r="G62" s="23">
         <v>4.1493000000000002</v>
       </c>
       <c r="H62" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I62" s="10" t="s">
+      <c r="I62" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J62" s="10">
+      <c r="J62" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="19">
+      <c r="A63" s="16">
         <v>8729210</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="C63" s="12">
+      <c r="C63" s="27">
         <v>30.2133</v>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="27">
         <v>-85.878299999999996</v>
       </c>
-      <c r="E63" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F63" s="8">
+      <c r="E63" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F63" s="22">
         <v>0.52</v>
       </c>
-      <c r="G63" s="14">
+      <c r="G63" s="23">
         <v>4.9870000000000001</v>
       </c>
       <c r="H63" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I63" s="10" t="s">
+      <c r="I63" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J63" s="10">
+      <c r="J63" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" s="11">
+      <c r="A64" s="10">
         <v>8729840</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C64" s="12">
+      <c r="C64" s="27">
         <v>30.404399999999999</v>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="27">
         <v>-87.211200000000005</v>
       </c>
-      <c r="E64" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F64" s="8">
+      <c r="E64" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F64" s="22">
         <v>0.51531163999999996</v>
       </c>
-      <c r="G64" s="9">
+      <c r="G64" s="23">
         <v>4.0664999999999996</v>
       </c>
       <c r="H64" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I64" s="10" t="s">
+      <c r="I64" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J64" s="10">
+      <c r="J64" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" s="11">
+      <c r="A65" s="10">
         <v>8735180</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C65" s="12">
+      <c r="C65" s="27">
         <v>30.25</v>
       </c>
-      <c r="D65" s="12">
+      <c r="D65" s="27">
         <v>-88.075000000000003</v>
       </c>
-      <c r="E65" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F65" s="8">
+      <c r="E65" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F65" s="22">
         <v>0.51468000000000003</v>
       </c>
-      <c r="G65" s="9">
+      <c r="G65" s="23">
         <v>5.0125999999999999</v>
       </c>
       <c r="H65" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I65" s="10" t="s">
+      <c r="I65" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J65" s="10">
+      <c r="J65" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="66" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="19">
+      <c r="A66" s="16">
         <v>8747437</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C66" s="9">
+      <c r="C66" s="23">
         <v>30.3263888888888</v>
       </c>
-      <c r="D66" s="9">
+      <c r="D66" s="23">
         <v>-89.325777777777702</v>
       </c>
-      <c r="E66" s="9">
+      <c r="E66" s="23">
         <v>0.44700000000000001</v>
       </c>
-      <c r="F66" s="9">
+      <c r="F66" s="23">
         <v>0.52116000000000007</v>
       </c>
-      <c r="G66" s="9">
+      <c r="G66" s="23">
         <v>4.7241</v>
       </c>
       <c r="H66" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I66" s="10" t="s">
+      <c r="I66" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J66" s="14">
+      <c r="J66" s="11">
         <v>-6</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" s="11">
+      <c r="A67" s="10">
         <v>8761724</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C67" s="12">
+      <c r="C67" s="27">
         <v>29.2633333333333</v>
       </c>
-      <c r="D67" s="12">
+      <c r="D67" s="27">
         <v>-89.956666666666607</v>
       </c>
-      <c r="E67" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F67" s="8">
+      <c r="E67" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F67" s="22">
         <v>0.51292000000000004</v>
       </c>
-      <c r="G67" s="9">
+      <c r="G67" s="23">
         <v>8.3241999999999994</v>
       </c>
       <c r="H67" s="7">
         <v>2009.5</v>
       </c>
-      <c r="I67" s="10" t="s">
+      <c r="I67" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J67" s="10">
+      <c r="J67" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" s="15">
+      <c r="A68" s="12">
         <v>8770613</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C68" s="12">
+      <c r="C68" s="27">
         <v>29.681699999999999</v>
       </c>
-      <c r="D68" s="12">
+      <c r="D68" s="27">
         <v>-94.984999999999999</v>
       </c>
-      <c r="E68" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F68" s="8">
+      <c r="E68" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F68" s="22">
         <v>0.52</v>
       </c>
-      <c r="G68" s="9">
+      <c r="G68" s="23">
         <v>4.1534000000000004</v>
       </c>
       <c r="H68" s="7">
         <v>1999.5</v>
       </c>
-      <c r="I68" s="10" t="s">
+      <c r="I68" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J68" s="10">
+      <c r="J68" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" s="15">
+      <c r="A69" s="12">
         <v>8771013</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C69" s="12">
+      <c r="C69" s="27">
         <v>29.48</v>
       </c>
-      <c r="D69" s="12">
+      <c r="D69" s="27">
         <v>-94.918300000000002</v>
       </c>
-      <c r="E69" s="8">
+      <c r="E69" s="22">
         <v>0.88</v>
       </c>
-      <c r="F69" s="8">
+      <c r="F69" s="22">
         <v>0.51</v>
       </c>
-      <c r="G69" s="9">
+      <c r="G69" s="23">
         <v>13.430400000000001</v>
       </c>
       <c r="H69" s="7">
         <v>1999.5</v>
       </c>
-      <c r="I69" s="10" t="s">
+      <c r="I69" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J69" s="10">
+      <c r="J69" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" s="19">
+      <c r="A70" s="16">
         <v>8771450</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C70" s="12">
+      <c r="C70" s="27">
         <v>29.31</v>
       </c>
-      <c r="D70" s="12">
+      <c r="D70" s="27">
         <v>-94.793300000000002</v>
       </c>
-      <c r="E70" s="8">
+      <c r="E70" s="22">
         <v>0.79051219512195137</v>
       </c>
-      <c r="F70" s="8">
+      <c r="F70" s="22">
         <v>0.51716000000000006</v>
       </c>
-      <c r="G70" s="9">
+      <c r="G70" s="23">
         <v>7.3090999999999999</v>
       </c>
       <c r="H70" s="7">
         <v>1999.5</v>
       </c>
-      <c r="I70" s="10" t="s">
+      <c r="I70" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J70" s="10">
+      <c r="J70" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A71" s="19">
+      <c r="A71" s="16">
         <v>8774770</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C71" s="12">
+      <c r="C71" s="27">
         <v>28.021699999999999</v>
       </c>
-      <c r="D71" s="12">
+      <c r="D71" s="27">
         <v>-97.046700000000001</v>
       </c>
-      <c r="E71" s="8">
+      <c r="E71" s="22">
         <v>0.55973170731707345</v>
       </c>
-      <c r="F71" s="8">
+      <c r="F71" s="22">
         <v>0.50444</v>
       </c>
-      <c r="G71" s="9">
+      <c r="G71" s="23">
         <v>8.3969000000000005</v>
       </c>
       <c r="H71" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I71" s="10" t="s">
+      <c r="I71" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J71" s="10">
+      <c r="J71" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A72" s="19">
+      <c r="A72" s="16">
         <v>8779770</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C72" s="12">
+      <c r="C72" s="27">
         <v>26.06</v>
       </c>
-      <c r="D72" s="12">
+      <c r="D72" s="27">
         <v>-97.215000000000003</v>
       </c>
-      <c r="E72" s="8">
+      <c r="E72" s="22">
         <v>0.34388312195121951</v>
       </c>
-      <c r="F72" s="8">
+      <c r="F72" s="22">
         <v>0.51673247999999994</v>
       </c>
-      <c r="G72" s="9">
+      <c r="G72" s="23">
         <v>5.9829999999999997</v>
       </c>
       <c r="H72" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I72" s="10" t="s">
+      <c r="I72" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J72" s="10">
+      <c r="J72" s="9">
         <v>-6</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A73" s="11">
+      <c r="A73" s="10">
         <v>9410170</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C73" s="12">
+      <c r="C73" s="27">
         <v>32.714190000000002</v>
       </c>
-      <c r="D73" s="12">
+      <c r="D73" s="27">
         <v>-117.173583333227</v>
       </c>
-      <c r="E73" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F73" s="8">
+      <c r="E73" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F73" s="22">
         <v>0.56979196000000032</v>
       </c>
-      <c r="G73" s="9">
+      <c r="G73" s="23">
         <v>2.6145</v>
       </c>
       <c r="H73" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I73" s="10" t="s">
+      <c r="I73" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J73" s="10">
+      <c r="J73" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A74" s="19">
+      <c r="A74" s="16">
         <v>9410230</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C74" s="12">
+      <c r="C74" s="27">
         <v>32.866700000000002</v>
       </c>
-      <c r="D74" s="12">
+      <c r="D74" s="27">
         <v>-117.258</v>
       </c>
-      <c r="E74" s="8">
+      <c r="E74" s="22">
         <v>0.50989034146341483</v>
       </c>
-      <c r="F74" s="8">
+      <c r="F74" s="22">
         <v>0.56497024000000007</v>
       </c>
-      <c r="G74" s="9">
+      <c r="G74" s="23">
         <v>1.7813000000000001</v>
       </c>
       <c r="H74" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I74" s="10" t="s">
+      <c r="I74" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J74" s="10">
+      <c r="J74" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" s="11">
+      <c r="A75" s="10">
         <v>9410660</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C75" s="12">
+      <c r="C75" s="27">
         <v>33.72</v>
       </c>
-      <c r="D75" s="12">
+      <c r="D75" s="27">
         <v>-118.27200000000001</v>
       </c>
-      <c r="E75" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F75" s="8">
+      <c r="E75" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F75" s="22">
         <v>0.56695156000000013</v>
       </c>
-      <c r="G75" s="9">
+      <c r="G75" s="23">
         <v>1.7181</v>
       </c>
       <c r="H75" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I75" s="10" t="s">
+      <c r="I75" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J75" s="10">
+      <c r="J75" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A76" s="11">
+      <c r="A76" s="10">
         <v>9410840</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C76" s="12">
+      <c r="C76" s="27">
         <v>34.008299999999998</v>
       </c>
-      <c r="D76" s="12">
+      <c r="D76" s="27">
         <v>-118.5</v>
       </c>
-      <c r="E76" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F76" s="8">
+      <c r="E76" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F76" s="22">
         <v>0.56612000000000018</v>
       </c>
-      <c r="G76" s="9">
+      <c r="G76" s="23">
         <v>1.4255</v>
       </c>
       <c r="H76" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I76" s="10" t="s">
+      <c r="I76" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J76" s="10">
+      <c r="J76" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A77" s="11">
+      <c r="A77" s="10">
         <v>9412110</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C77" s="12">
+      <c r="C77" s="27">
         <v>35.176699999999997</v>
       </c>
-      <c r="D77" s="12">
+      <c r="D77" s="27">
         <v>-120.76</v>
       </c>
-      <c r="E77" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F77" s="8">
+      <c r="E77" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F77" s="22">
         <v>0.56492000000000009</v>
       </c>
-      <c r="G77" s="9">
+      <c r="G77" s="23">
         <v>0.98040000000000005</v>
       </c>
       <c r="H77" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I77" s="10" t="s">
+      <c r="I77" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J77" s="10">
+      <c r="J77" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A78" s="20">
+      <c r="A78" s="17">
         <v>9413450</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C78" s="12">
+      <c r="C78" s="27">
         <v>36.604999999999997</v>
       </c>
-      <c r="D78" s="12">
+      <c r="D78" s="27">
         <v>-121.88800000000001</v>
       </c>
-      <c r="E78" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F78" s="8">
+      <c r="E78" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F78" s="22">
         <v>0.56503999999999999</v>
       </c>
-      <c r="G78" s="9">
+      <c r="G78" s="23">
         <v>1.1143000000000001</v>
       </c>
       <c r="H78" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I78" s="10" t="s">
+      <c r="I78" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J78" s="10">
+      <c r="J78" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A79" s="16">
+      <c r="A79" s="13">
         <v>9414290</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C79" s="12">
+      <c r="C79" s="27">
         <v>37.806694444444403</v>
       </c>
-      <c r="D79" s="12">
+      <c r="D79" s="27">
         <v>-122.465</v>
       </c>
-      <c r="E79" s="8">
+      <c r="E79" s="22">
         <v>0.35387934146341471</v>
       </c>
-      <c r="F79" s="8">
+      <c r="F79" s="22">
         <v>0.5712106800000003</v>
       </c>
-      <c r="G79" s="9">
+      <c r="G79" s="23">
         <v>1.7281</v>
       </c>
       <c r="H79" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I79" s="10" t="s">
+      <c r="I79" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J79" s="10">
+      <c r="J79" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A80" s="20">
+      <c r="A80" s="17">
         <v>9414750</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C80" s="12">
+      <c r="C80" s="27">
         <v>37.771666666666597</v>
       </c>
-      <c r="D80" s="12">
+      <c r="D80" s="27">
         <v>-122.29833333333301</v>
       </c>
-      <c r="E80" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F80" s="8">
+      <c r="E80" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F80" s="22">
         <v>0.58041039999999988</v>
       </c>
-      <c r="G80" s="9">
+      <c r="G80" s="23">
         <v>0.94879999999999998</v>
       </c>
       <c r="H80" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I80" s="10" t="s">
+      <c r="I80" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J80" s="10">
+      <c r="J80" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A81" s="20">
+      <c r="A81" s="17">
         <v>9415020</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C81" s="12">
+      <c r="C81" s="27">
         <v>37.996099999999998</v>
       </c>
-      <c r="D81" s="12">
+      <c r="D81" s="27">
         <v>-122.97669999999999</v>
       </c>
-      <c r="E81" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F81" s="8">
+      <c r="E81" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F81" s="22">
         <v>0.57032000000000016</v>
       </c>
-      <c r="G81" s="9">
+      <c r="G81" s="23">
         <v>1.5385</v>
       </c>
       <c r="H81" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I81" s="10" t="s">
+      <c r="I81" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J81" s="10">
+      <c r="J81" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A82" s="20">
+      <c r="A82" s="17">
         <v>9415144</v>
       </c>
       <c r="B82" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C82" s="12">
+      <c r="C82" s="27">
         <v>38.055999999999997</v>
       </c>
-      <c r="D82" s="12">
+      <c r="D82" s="27">
         <v>-122.0395</v>
       </c>
-      <c r="E82" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F82" s="8">
+      <c r="E82" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F82" s="22">
         <v>0.55991367999999975</v>
       </c>
-      <c r="G82" s="9">
+      <c r="G82" s="23">
         <v>1.2411000000000001</v>
       </c>
       <c r="H82" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I82" s="10" t="s">
+      <c r="I82" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J82" s="10">
+      <c r="J82" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A83" s="20">
+      <c r="A83" s="17">
         <v>9416841</v>
       </c>
       <c r="B83" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C83" s="12">
+      <c r="C83" s="27">
         <v>38.9133</v>
       </c>
-      <c r="D83" s="12">
+      <c r="D83" s="27">
         <v>-123.708</v>
       </c>
-      <c r="E83" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F83" s="8">
+      <c r="E83" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F83" s="22">
         <v>0.57148000000000021</v>
       </c>
-      <c r="G83" s="9">
+      <c r="G83" s="23">
         <v>1.1508</v>
       </c>
       <c r="H83" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I83" s="10" t="s">
+      <c r="I83" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J83" s="10">
+      <c r="J83" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A84" s="16">
+      <c r="A84" s="13">
         <v>9418767</v>
       </c>
       <c r="B84" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C84" s="12">
+      <c r="C84" s="27">
         <v>40.7667</v>
       </c>
-      <c r="D84" s="12">
+      <c r="D84" s="27">
         <v>-124.217</v>
       </c>
-      <c r="E84" s="8">
+      <c r="E84" s="22">
         <v>0.56244502439024391</v>
       </c>
-      <c r="F84" s="8">
+      <c r="F84" s="22">
         <v>0.58359976000000024</v>
       </c>
-      <c r="G84" s="9">
+      <c r="G84" s="23">
         <v>4.7328999999999999</v>
       </c>
       <c r="H84" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I84" s="10" t="s">
+      <c r="I84" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J84" s="10">
+      <c r="J84" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A85" s="20">
+      <c r="A85" s="17">
         <v>9431647</v>
       </c>
       <c r="B85" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C85" s="12">
+      <c r="C85" s="27">
         <v>42.738970000000002</v>
       </c>
-      <c r="D85" s="12">
+      <c r="D85" s="27">
         <v>-124.49827777756499</v>
       </c>
-      <c r="E85" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F85" s="8">
+      <c r="E85" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F85" s="22">
         <v>0.58884000000000025</v>
       </c>
-      <c r="G85" s="9">
+      <c r="G85" s="23">
         <v>-6.8999999999999999E-3</v>
       </c>
       <c r="H85" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I85" s="10" t="s">
+      <c r="I85" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J85" s="10">
+      <c r="J85" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A86" s="20">
+      <c r="A86" s="17">
         <v>9432780</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C86" s="12">
+      <c r="C86" s="27">
         <v>43.344999999999999</v>
       </c>
-      <c r="D86" s="12">
+      <c r="D86" s="27">
         <v>-124.322</v>
       </c>
-      <c r="E86" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F86" s="8">
+      <c r="E86" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F86" s="22">
         <v>0.59291999999999989</v>
       </c>
-      <c r="G86" s="9">
+      <c r="G86" s="23">
         <v>0.70369999999999999</v>
       </c>
       <c r="H86" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I86" s="10" t="s">
+      <c r="I86" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J86" s="10">
+      <c r="J86" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A87" s="16">
+      <c r="A87" s="13">
         <v>9435380</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C87" s="12">
+      <c r="C87" s="27">
         <v>44.625</v>
       </c>
-      <c r="D87" s="12">
+      <c r="D87" s="27">
         <v>-124.04300000000001</v>
       </c>
-      <c r="E87" s="8">
+      <c r="E87" s="22">
         <v>1.1155365853658537</v>
       </c>
-      <c r="F87" s="8">
+      <c r="F87" s="22">
         <v>0.60172000000000025</v>
       </c>
-      <c r="G87" s="9">
+      <c r="G87" s="23">
         <v>2.0605000000000002</v>
       </c>
       <c r="H87" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I87" s="10" t="s">
+      <c r="I87" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J87" s="10">
+      <c r="J87" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A88" s="16">
+      <c r="A88" s="13">
         <v>9440910</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C88" s="12">
+      <c r="C88" s="27">
         <v>46.707470000000001</v>
       </c>
-      <c r="D88" s="12">
+      <c r="D88" s="27">
         <v>-123.96691666666</v>
       </c>
-      <c r="E88" s="8">
+      <c r="E88" s="22">
         <v>0.63419453658536584</v>
       </c>
-      <c r="F88" s="8">
+      <c r="F88" s="22">
         <v>0.60877856000000019</v>
       </c>
-      <c r="G88" s="9">
+      <c r="G88" s="23">
         <v>-0.28749999999999998</v>
       </c>
       <c r="H88" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I88" s="10" t="s">
+      <c r="I88" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J88" s="10">
+      <c r="J88" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A89" s="20">
+      <c r="A89" s="17">
         <v>9444090</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C89" s="12">
+      <c r="C89" s="27">
         <v>48.125</v>
       </c>
-      <c r="D89" s="12">
+      <c r="D89" s="27">
         <v>-123.44</v>
       </c>
-      <c r="E89" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F89" s="8">
+      <c r="E89" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F89" s="22">
         <v>0.58612143999999988</v>
       </c>
-      <c r="G89" s="9">
+      <c r="G89" s="23">
         <v>0.2271</v>
       </c>
       <c r="H89" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I89" s="10" t="s">
+      <c r="I89" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J89" s="10">
+      <c r="J89" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A90" s="16">
+      <c r="A90" s="13">
         <v>9444900</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C90" s="12">
+      <c r="C90" s="27">
         <v>48.111699999999999</v>
       </c>
-      <c r="D90" s="12">
+      <c r="D90" s="27">
         <v>-122.758</v>
       </c>
-      <c r="E90" s="8">
+      <c r="E90" s="22">
         <v>0.90963256097560974</v>
       </c>
-      <c r="F90" s="8">
+      <c r="F90" s="22">
         <v>0.60385860000000013</v>
       </c>
-      <c r="G90" s="9">
+      <c r="G90" s="23">
         <v>1.45</v>
       </c>
       <c r="H90" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I90" s="10" t="s">
+      <c r="I90" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J90" s="10">
+      <c r="J90" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A91" s="16">
+      <c r="A91" s="13">
         <v>9447130</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C91" s="12">
+      <c r="C91" s="27">
         <v>47.602638888888798</v>
       </c>
-      <c r="D91" s="12">
+      <c r="D91" s="27">
         <v>-122.339305555555</v>
       </c>
-      <c r="E91" s="8">
+      <c r="E91" s="22">
         <v>0.65365465853658566</v>
       </c>
-      <c r="F91" s="8">
+      <c r="F91" s="22">
         <v>0.63848795999999997</v>
       </c>
-      <c r="G91" s="9">
+      <c r="G91" s="23">
         <v>2.1997</v>
       </c>
       <c r="H91" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I91" s="10" t="s">
+      <c r="I91" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J91" s="10">
+      <c r="J91" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A92" s="20">
+      <c r="A92" s="17">
         <v>9449424</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C92" s="12">
+      <c r="C92" s="27">
         <v>48.863300000000002</v>
       </c>
-      <c r="D92" s="12">
+      <c r="D92" s="27">
         <v>-122.758</v>
       </c>
-      <c r="E92" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F92" s="8">
+      <c r="E92" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F92" s="22">
         <v>0.61152000000000006</v>
       </c>
-      <c r="G92" s="9">
+      <c r="G92" s="23">
         <v>-0.43369999999999997</v>
       </c>
       <c r="H92" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I92" s="10" t="s">
+      <c r="I92" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J92" s="10">
+      <c r="J92" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A93" s="20">
+      <c r="A93" s="17">
         <v>9449880</v>
       </c>
       <c r="B93" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C93" s="12">
+      <c r="C93" s="27">
         <v>48.546666666666603</v>
       </c>
-      <c r="D93" s="12">
+      <c r="D93" s="27">
         <v>-123.01</v>
       </c>
-      <c r="E93" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F93" s="8">
+      <c r="E93" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F93" s="22">
         <v>0.59454636000000027</v>
       </c>
-      <c r="G93" s="9">
+      <c r="G93" s="23">
         <v>1.2426999999999999</v>
       </c>
       <c r="H93" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I93" s="10" t="s">
+      <c r="I93" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J93" s="10">
+      <c r="J93" s="9">
         <v>-8</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A94" s="20">
+      <c r="A94" s="17">
         <v>9751401</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C94" s="12">
+      <c r="C94" s="27">
         <v>17.6947222222222</v>
       </c>
-      <c r="D94" s="12">
+      <c r="D94" s="27">
         <v>-64.753805555555502</v>
       </c>
-      <c r="E94" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F94" s="8">
+      <c r="E94" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F94" s="22">
         <v>0.50864000000000009</v>
       </c>
-      <c r="G94" s="9">
+      <c r="G94" s="23">
         <v>3.0421999999999998</v>
       </c>
       <c r="H94" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I94" s="10" t="s">
+      <c r="I94" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="J94" s="10">
+      <c r="J94" s="9">
         <v>-4</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A95" s="20">
+      <c r="A95" s="17">
         <v>9751639</v>
       </c>
       <c r="B95" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C95" s="12">
+      <c r="C95" s="27">
         <v>18.335833333333301</v>
       </c>
-      <c r="D95" s="12">
+      <c r="D95" s="27">
         <v>-64.92</v>
       </c>
-      <c r="E95" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F95" s="8">
+      <c r="E95" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F95" s="22">
         <v>0.50960000000000005</v>
       </c>
-      <c r="G95" s="9">
+      <c r="G95" s="23">
         <v>2.4573</v>
       </c>
       <c r="H95" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I95" s="10" t="s">
+      <c r="I95" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="J95" s="10">
+      <c r="J95" s="9">
         <v>-4</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A96" s="20">
+      <c r="A96" s="17">
         <v>9755371</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C96" s="12">
+      <c r="C96" s="27">
         <v>18.458939999999998</v>
       </c>
-      <c r="D96" s="12">
+      <c r="D96" s="27">
         <v>-66.116416666242799</v>
       </c>
-      <c r="E96" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F96" s="8">
+      <c r="E96" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F96" s="22">
         <v>0.51919999999999999</v>
       </c>
-      <c r="G96" s="9">
+      <c r="G96" s="23">
         <v>2.6259999999999999</v>
       </c>
       <c r="H96" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I96" s="10" t="s">
+      <c r="I96" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="J96" s="10">
+      <c r="J96" s="9">
         <v>-4</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A97" s="20">
+      <c r="A97" s="17">
         <v>9759110</v>
       </c>
       <c r="B97" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C97" s="12">
+      <c r="C97" s="27">
         <v>17.970079999999999</v>
       </c>
-      <c r="D97" s="12">
+      <c r="D97" s="27">
         <v>-67.046416666242806</v>
       </c>
-      <c r="E97" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F97" s="8">
+      <c r="E97" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F97" s="22">
         <v>0.50814855999999997</v>
       </c>
-      <c r="G97" s="9">
+      <c r="G97" s="23">
         <v>2.4704999999999999</v>
       </c>
       <c r="H97" s="7">
         <v>1992.5</v>
       </c>
-      <c r="I97" s="10" t="s">
+      <c r="I97" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="J97" s="10">
+      <c r="J97" s="9">
         <v>-4</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A98" s="10">
+      <c r="A98" s="9">
         <v>9450460</v>
       </c>
       <c r="B98" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C98" s="8">
+      <c r="C98" s="22">
         <v>55.331829999999997</v>
       </c>
-      <c r="D98" s="8">
+      <c r="D98" s="22">
         <v>-131.626194444232</v>
       </c>
-      <c r="E98" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F98" s="8">
+      <c r="E98" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F98" s="22">
         <v>0.68831431999999992</v>
       </c>
-      <c r="G98" s="8">
+      <c r="G98" s="22">
         <v>-2.1034000000000002</v>
       </c>
-      <c r="H98" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I98" s="10" t="s">
+      <c r="H98" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I98" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J98" s="10">
+      <c r="J98" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A99" s="10">
+      <c r="A99" s="9">
         <v>9451600</v>
       </c>
       <c r="B99" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C99" s="8">
+      <c r="C99" s="22">
         <v>57.051699999999997</v>
       </c>
-      <c r="D99" s="8">
+      <c r="D99" s="22">
         <v>-135.34200000000001</v>
       </c>
-      <c r="E99" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F99" s="8">
+      <c r="E99" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F99" s="22">
         <v>0.62114012000000018</v>
       </c>
-      <c r="G99" s="8">
+      <c r="G99" s="22">
         <v>-5.4402999999999997</v>
       </c>
-      <c r="H99" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I99" s="10" t="s">
+      <c r="H99" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I99" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J99" s="10">
+      <c r="J99" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A100" s="10">
+      <c r="A100" s="9">
         <v>9452210</v>
       </c>
       <c r="B100" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C100" s="8">
+      <c r="C100" s="22">
         <v>58.298299999999998</v>
       </c>
-      <c r="D100" s="8">
+      <c r="D100" s="22">
         <v>-134.41200000000001</v>
       </c>
-      <c r="E100" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F100" s="8">
+      <c r="E100" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F100" s="22">
         <v>0.69884000000000057</v>
       </c>
-      <c r="G100" s="8">
+      <c r="G100" s="22">
         <v>-16.8264</v>
       </c>
-      <c r="H100" s="24">
+      <c r="H100" s="21">
         <v>2009.5</v>
       </c>
-      <c r="I100" s="10" t="s">
+      <c r="I100" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J100" s="10">
+      <c r="J100" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A101" s="10">
+      <c r="A101" s="9">
         <v>9452400</v>
       </c>
       <c r="B101" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C101" s="8">
+      <c r="C101" s="22">
         <v>59.45</v>
       </c>
-      <c r="D101" s="8">
+      <c r="D101" s="22">
         <v>-135.327</v>
       </c>
-      <c r="E101" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F101" s="8">
+      <c r="E101" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F101" s="22">
         <v>0.70404</v>
       </c>
-      <c r="G101" s="8">
+      <c r="G101" s="22">
         <v>-23.262</v>
       </c>
-      <c r="H101" s="24">
+      <c r="H101" s="21">
         <v>2009.5</v>
       </c>
-      <c r="I101" s="10" t="s">
+      <c r="I101" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J101" s="10">
+      <c r="J101" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A102" s="10">
+      <c r="A102" s="9">
         <v>9453220</v>
       </c>
       <c r="B102" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C102" s="8">
+      <c r="C102" s="22">
         <v>59.548499999999997</v>
       </c>
-      <c r="D102" s="8">
+      <c r="D102" s="22">
         <v>-139.73339999999999</v>
       </c>
-      <c r="E102" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F102" s="8">
+      <c r="E102" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F102" s="22">
         <v>0.62280000000000024</v>
       </c>
       <c r="G102" s="25">
         <v>-19.203499999999998</v>
       </c>
-      <c r="H102" s="24">
+      <c r="H102" s="21">
         <v>2009.5</v>
       </c>
-      <c r="I102" s="10" t="s">
+      <c r="I102" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J102" s="10">
+      <c r="J102" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A103" s="10">
+      <c r="A103" s="9">
         <v>9454050</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="C103" s="8">
+      <c r="C103" s="22">
         <v>60.558300000000003</v>
       </c>
-      <c r="D103" s="8">
+      <c r="D103" s="22">
         <v>-145.75299999999999</v>
       </c>
-      <c r="E103" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F103" s="8">
+      <c r="E103" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F103" s="22">
         <v>0.65350887999999951</v>
       </c>
-      <c r="G103" s="8">
+      <c r="G103" s="22">
         <v>-2.5718999999999999</v>
       </c>
-      <c r="H103" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I103" s="10" t="s">
+      <c r="H103" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I103" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J103" s="10">
+      <c r="J103" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A104" s="10">
+      <c r="A104" s="9">
         <v>9454240</v>
       </c>
       <c r="B104" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C104" s="8">
+      <c r="C104" s="22">
         <v>61.125</v>
       </c>
-      <c r="D104" s="8">
+      <c r="D104" s="22">
         <v>-146.36199999999999</v>
       </c>
-      <c r="E104" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F104" s="8">
+      <c r="E104" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F104" s="22">
         <v>0.64807871999999955</v>
       </c>
-      <c r="G104" s="8">
+      <c r="G104" s="22">
         <v>-10.3459</v>
       </c>
-      <c r="H104" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I104" s="10" t="s">
+      <c r="H104" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I104" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J104" s="10">
+      <c r="J104" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A105" s="10">
+      <c r="A105" s="9">
         <v>9455090</v>
       </c>
       <c r="B105" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C105" s="8">
+      <c r="C105" s="22">
         <v>60.12</v>
       </c>
-      <c r="D105" s="8">
+      <c r="D105" s="22">
         <v>-149.42666666666599</v>
       </c>
-      <c r="E105" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F105" s="8">
+      <c r="E105" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F105" s="22">
         <v>0.62956000000000012</v>
       </c>
-      <c r="G105" s="8">
+      <c r="G105" s="22">
         <v>-6.4725999999999999</v>
       </c>
-      <c r="H105" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I105" s="10" t="s">
+      <c r="H105" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I105" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J105" s="10">
+      <c r="J105" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A106" s="10">
+      <c r="A106" s="9">
         <v>9455500</v>
       </c>
       <c r="B106" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="C106" s="8">
+      <c r="C106" s="22">
         <v>59.440527777777703</v>
       </c>
-      <c r="D106" s="8">
+      <c r="D106" s="22">
         <v>-151.719944444444</v>
       </c>
-      <c r="E106" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F106" s="8">
+      <c r="E106" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F106" s="22">
         <v>0.71996000000000038</v>
       </c>
-      <c r="G106" s="8">
+      <c r="G106" s="22">
         <v>-8.1096000000000004</v>
       </c>
-      <c r="H106" s="24">
+      <c r="H106" s="21">
         <v>2009.5</v>
       </c>
-      <c r="I106" s="10" t="s">
+      <c r="I106" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J106" s="10">
+      <c r="J106" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A107" s="10">
+      <c r="A107" s="9">
         <v>9455760</v>
       </c>
       <c r="B107" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="C107" s="8">
+      <c r="C107" s="22">
         <v>60.683300000000003</v>
       </c>
-      <c r="D107" s="8">
+      <c r="D107" s="22">
         <v>-151.398</v>
       </c>
-      <c r="E107" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F107" s="8">
+      <c r="E107" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F107" s="22">
         <v>0.75091999999999981</v>
       </c>
-      <c r="G107" s="8">
+      <c r="G107" s="22">
         <v>-11.367699999999999</v>
       </c>
-      <c r="H107" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I107" s="10" t="s">
+      <c r="H107" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I107" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J107" s="10">
+      <c r="J107" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A108" s="10">
+      <c r="A108" s="9">
         <v>9455920</v>
       </c>
       <c r="B108" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C108" s="8">
+      <c r="C108" s="22">
         <v>61.238305555555499</v>
       </c>
-      <c r="D108" s="8">
+      <c r="D108" s="22">
         <v>-149.88999999999999</v>
       </c>
-      <c r="E108" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F108" s="8">
+      <c r="E108" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F108" s="22">
         <v>0.85556000000000054</v>
       </c>
-      <c r="G108" s="8">
+      <c r="G108" s="22">
         <v>-6.8033999999999999</v>
       </c>
-      <c r="H108" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I108" s="10" t="s">
+      <c r="H108" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I108" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J108" s="10">
+      <c r="J108" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A109" s="10">
+      <c r="A109" s="9">
         <v>9457292</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C109" s="8">
+      <c r="C109" s="22">
         <v>57.731699999999996</v>
       </c>
-      <c r="D109" s="8">
+      <c r="D109" s="22">
         <v>-152.512</v>
       </c>
-      <c r="E109" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F109" s="8">
+      <c r="E109" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F109" s="22">
         <v>0.60700000000000021</v>
       </c>
-      <c r="G109" s="8">
+      <c r="G109" s="22">
         <v>-8.2149999999999999</v>
       </c>
-      <c r="H109" s="24">
+      <c r="H109" s="21">
         <v>2009.5</v>
       </c>
-      <c r="I109" s="10" t="s">
+      <c r="I109" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J109" s="10">
+      <c r="J109" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A110" s="10">
+      <c r="A110" s="9">
         <v>9459450</v>
       </c>
       <c r="B110" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="C110" s="8">
+      <c r="C110" s="22">
         <v>55.336694444444397</v>
       </c>
-      <c r="D110" s="8">
+      <c r="D110" s="22">
         <v>-160.50200000000001</v>
       </c>
-      <c r="E110" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F110" s="8">
+      <c r="E110" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F110" s="22">
         <v>0.5881737600000001</v>
       </c>
-      <c r="G110" s="8">
+      <c r="G110" s="22">
         <v>4.0441000000000003</v>
       </c>
-      <c r="H110" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I110" s="10" t="s">
+      <c r="H110" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I110" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J110" s="10">
+      <c r="J110" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A111" s="10">
+      <c r="A111" s="9">
         <v>9461380</v>
       </c>
       <c r="B111" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C111" s="8">
+      <c r="C111" s="22">
         <v>51.863300000000002</v>
       </c>
-      <c r="D111" s="8">
+      <c r="D111" s="22">
         <v>-176.63200000000001</v>
       </c>
-      <c r="E111" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F111" s="8">
+      <c r="E111" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F111" s="22">
         <v>0.54522104000000016</v>
       </c>
-      <c r="G111" s="8">
+      <c r="G111" s="22">
         <v>-0.69830000000000003</v>
       </c>
-      <c r="H111" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I111" s="10" t="s">
+      <c r="H111" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I111" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J111" s="10">
+      <c r="J111" s="9">
         <v>-10</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A112" s="10">
+      <c r="A112" s="9">
         <v>9462620</v>
       </c>
       <c r="B112" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C112" s="8">
+      <c r="C112" s="22">
         <v>53.88</v>
       </c>
-      <c r="D112" s="8">
+      <c r="D112" s="22">
         <v>-166.53700000000001</v>
       </c>
-      <c r="E112" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F112" s="8">
+      <c r="E112" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F112" s="22">
         <v>0.54391999999999996</v>
       </c>
-      <c r="G112" s="8">
+      <c r="G112" s="22">
         <v>0.85419999999999996</v>
       </c>
-      <c r="H112" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I112" s="10" t="s">
+      <c r="H112" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I112" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J112" s="10">
+      <c r="J112" s="9">
         <v>-9</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A113" s="10">
+      <c r="A113" s="9">
         <v>9463502</v>
       </c>
       <c r="B113" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="C113" s="8">
+      <c r="C113" s="22">
         <v>55.99</v>
       </c>
-      <c r="D113" s="8">
+      <c r="D113" s="22">
         <v>-160.56200000000001</v>
       </c>
-      <c r="E113" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F113" s="8">
+      <c r="E113" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F113" s="22">
         <v>0.62695999999999996</v>
       </c>
-      <c r="G113" s="10">
+      <c r="G113" s="22">
         <v>9.4748000000000001</v>
       </c>
-      <c r="H113" s="24">
-        <v>1992.5</v>
-      </c>
-      <c r="I113" s="10" t="s">
+      <c r="H113" s="21">
+        <v>1992.5</v>
+      </c>
+      <c r="I113" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="J113" s="10">
+      <c r="J113" s="9">
         <v>-9</v>
       </c>
     </row>

</xml_diff>